<commit_message>
Auto update govt jobs dashboard data
</commit_message>
<xml_diff>
--- a/jobs/government_jobs_tracker.xlsx
+++ b/jobs/government_jobs_tracker.xlsx
@@ -17,8 +17,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eligible Apply Now'!$A$1:$M$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Doubtful Manual Check'!$A$1:$M$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Avoid or Closed'!$A$1:$M$135</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All Raw Matches'!$A$1:$M$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Avoid or Closed'!$A$1:$M$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All Raw Matches'!$A$1:$M$147</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sources'!$A$1:$D$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Profile'!$A$1:$B$10</definedName>
   </definedNames>
@@ -690,7 +690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M135"/>
+  <dimension ref="A1:M146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1348,7 +1348,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Regular)-2025 Advt.No.-01/2026 (02-07-2026)</t>
+          <t>Press release and written result of the Recruitment of Forest Range Officer,Advt.No.-04/2024 (03-07-2026)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1358,17 +1358,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>02-07-2026</t>
+          <t>03-07-2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>02-07-2026</t>
+          <t>03-07-2026</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_and_P.T_Result_01_26_dated_02_07_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_and_Written_Result_04_24_dated_03_07_2026.pdf</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1406,44 +1406,44 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Regular)-2025 Advt.No.-01/2026 (02-07-2026)</t>
+          <t>Press release and written result of the Recruitment of Forest Range Officer,Advt.No.-04/2024 (03-07-2026)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Press release and written result of the Recruitment of Forest Range Officer,Advt.No.-04/2024 (03-07-2026)</t>
+          <t>Examination | Combined State/Upper Subordinate Services Examination | | A-1/E-1/2026 , 25/06/2026 | 25/06/2026 | 27/07/2026 | 27/07/2026 | 03/08/2026 | 25/06/2026 03/08/2026 | User</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>03-07-2026</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>03-07-2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_and_Written_Result_04_24_dated_03_07_2026.pdf</t>
+          <t>https://uppsc.up.nic.in/OuterPages/UserHelp.aspx?ID=114</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Uttar Pradesh</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>JPSC</t>
+          <t>UPPSC</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1461,54 +1461,54 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/</t>
+          <t>https://uppsc.up.nic.in/CandidatePages/Notifications.aspx</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Press release and written result of the Recruitment of Forest Range Officer,Advt.No.-04/2024 (03-07-2026)</t>
+          <t>Examination | Combined State/Upper Subordinate Services Examination | | A-1/E-1/2026 , 25/06/2026 | 25/06/2026 | 27/07/2026 | 27/07/2026 | 03/08/2026 | 25/06/2026 03/08/2026 | User Instructions | View Advertisement | Apply</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Examination | Combined State/Upper Subordinate Services Examination | | A-1/E-1/2026 , 25/06/2026 | 25/06/2026 | 27/07/2026 | 27/07/2026 | 03/08/2026 | 25/06/2026 03/08/2026 | User</t>
+          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 (06-07-2026)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Education/subject not clearly matched</t>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>06-07-2026</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>06-07-2026</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://uppsc.up.nic.in/OuterPages/UserHelp.aspx?ID=114</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_and_P.T_Result_05_26_dated_06_07_2026.pdf</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Uttar Pradesh</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>UPPSC</t>
+          <t>JPSC</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1526,44 +1526,44 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Education/subject not clearly matched</t>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>https://uppsc.up.nic.in/CandidatePages/Notifications.aspx</t>
+          <t>https://www.jpsc.gov.in/</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Examination | Combined State/Upper Subordinate Services Examination | | A-1/E-1/2026 , 25/06/2026 | 25/06/2026 | 27/07/2026 | 27/07/2026 | 03/08/2026 | 25/06/2026 03/08/2026 | User Instructions | View Advertisement | Apply</t>
+          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 (06-07-2026)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 (06-07-2026)</t>
+          <t>Press Release regarding Combined Civil Services Main Examination Uploaded date:-07-07-2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>06-07-2026</t>
+          <t>07-07-2026</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>06-07-2026</t>
+          <t>07-07-2026</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_and_P.T_Result_05_26_dated_06_07_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_05_26_dated_07_07_2026.pdf</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 (06-07-2026)</t>
+          <t>Press Release regarding Combined Civil Services Main Examination Uploaded date:-07-07-2026</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Press Release regarding Combined Civil Services Main Examination Uploaded date:-07-07-2026</t>
+          <t>Press release and written result of the Recruitment of Assistant Conservator of Forest,Advt.No.-03/2024 (07-07-2026)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_05_26_dated_07_07_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_and_Written_Result_03_24_dated_07_07_2026.pdf</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>General/Other</t>
+          <t>Office/Clerical</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1666,34 +1666,34 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Press Release regarding Combined Civil Services Main Examination Uploaded date:-07-07-2026</t>
+          <t>Press release and written result of the Recruitment of Assistant Conservator of Forest,Advt.No.-03/2024 (07-07-2026)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Press release and written result of the Recruitment of Assistant Conservator of Forest,Advt.No.-03/2024 (07-07-2026)</t>
+          <t>Press Release regarding Recruitment of Deputy Director, Prosecution Advt.No.-15/2023 Uploaded date:-08-12-2025</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Specific non-CSE subject appears required | Non-CSE subject risk: prosecution | Last date appears closed</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>07-07-2026</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>07-07-2026</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_and_Written_Result_03_24_dated_07_07_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_15_23_dated_08_12_2025.pdf</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Office/Clerical</t>
+          <t>General/Other</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: it  | Specific non-CSE subject appears required | Non-CSE subject risk: prosecution | Last date appears closed</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1731,34 +1731,34 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Press release and written result of the Recruitment of Assistant Conservator of Forest,Advt.No.-03/2024 (07-07-2026)</t>
+          <t>Press Release regarding Recruitment of Deputy Director, Prosecution Advt.No.-15/2023 Uploaded date:-08-12-2025</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Press Release regarding Recruitment of Deputy Director, Prosecution Advt.No.-15/2023 Uploaded date:-08-12-2025</t>
+          <t>Press release and Instructions regarding Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 uploaded date :09-05-2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Specific non-CSE subject appears required | Non-CSE subject risk: prosecution | Last date appears closed</t>
+          <t>Auto-extracted: Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-05-2026</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-05-2026</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_15_23_dated_08_12_2025.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_05_26_dated_09_05_2026.pdf</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Specific non-CSE subject appears required | Non-CSE subject risk: prosecution | Last date appears closed</t>
+          <t>Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1796,34 +1796,34 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Press Release regarding Recruitment of Deputy Director, Prosecution Advt.No.-15/2023 Uploaded date:-08-12-2025</t>
+          <t>Press release and Instructions regarding Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 uploaded date :09-05-2026</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Press release and Instructions regarding Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 uploaded date :09-05-2026</t>
+          <t>Press release regarding Jharkhand Combined Civil Services Examination, Advt.No.-01/2026, 05/2026 and 06/2026 (09-07-2026)</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>09-05-2026</t>
+          <t>09-07-2026</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>09-05-2026</t>
+          <t>09-07-2026</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_05_26_dated_09_05_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_06_26_dated_09_07_2026.pdf</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Education/subject not clearly matched | Last date appears closed</t>
+          <t>Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Press release and Instructions regarding Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 uploaded date :09-05-2026</t>
+          <t>Press release regarding Jharkhand Combined Civil Services Examination, Advt.No.-01/2026, 05/2026 and 06/2026 (09-07-2026)</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2648,7 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 01/2026, 02/2026 &amp; 04/</t>
+          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 02/2026 &amp; 04/2026 | 20</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2658,17 +2658,17 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-0506603f0071/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-23d707fe007d/publicNotice</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2706,34 +2706,34 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 01/2026, 02/2026 &amp; 04/2026 | 2026-06-26</t>
+          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 02/2026 &amp; 04/2026 | 2026-07-02</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 02/2026 &amp; 04/2026 | 20</t>
+          <t>NOTICE REGARDING DISPLAY OF OMR ANSWER SHEETS OF THE COMMON ELIGIBILITY TEST (CET)-2025 (GROUP-C) WRITTEN EXAMINATION IN CANDIDATE LOGIN OF ALL APPEARED CANDIDATES | 2026-07-04</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-23d707fe007d/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-2d7fabd90086/publicNotice</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -2771,34 +2771,34 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 02/2026 &amp; 04/2026 | 2026-07-02</t>
+          <t>NOTICE REGARDING DISPLAY OF OMR ANSWER SHEETS OF THE COMMON ELIGIBILITY TEST (CET)-2025 (GROUP-C) WRITTEN EXAMINATION IN CANDIDATE LOGIN OF ALL APPEARED CANDIDATES | 2026-07-04</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL SCREENING TEST (PST) FOR MALE CONSTABLE (GD) AND MALE CONSTABLE (GOVERNMENT RAILWAY POLICE) AGAINST ADVERTISEMENT NO. 01/2026, CATEGORY NO. 01</t>
+          <t>PUBLIC NOTICE REGARDING CONSIDERING CLOSING DATE OF SUBMISSION OF APPLICATION FORM FOR THE POST OF GROUP-D AGAINST ADVERTISEMENT NO. 05/2026. | 2026-07-07</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: ai, mis | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-237201a5007a/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-3cc194ce008c/publicNotice</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: ai, mis | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2836,34 +2836,34 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL SCREENING TEST (PST) FOR MALE CONSTABLE (GD) AND MALE CONSTABLE (GOVERNMENT RAILWAY POLICE) AGAINST ADVERTISEMENT NO. 01/2026, CATEGORY NO. 01 AND 03 OF POLICE DEPARTMENT, HARYANA. | 2026-07-02</t>
+          <t>PUBLIC NOTICE REGARDING CONSIDERING CLOSING DATE OF SUBMISSION OF APPLICATION FORM FOR THE POST OF GROUP-D AGAINST ADVERTISEMENT NO. 05/2026. | 2026-07-07</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>NOTICE REGARDING DISPLAY OF OMR ANSWER SHEETS OF THE COMMON ELIGIBILITY TEST (CET)-2025 (GROUP-C) WRITTEN EXAMINATION IN CANDIDATE LOGIN OF ALL APPEARED CANDIDATES | 2026-07-04</t>
+          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR VARIOUS POSTS AGAINST ADVERTISEMENT NO. 06/2026 OF PRISON DEPARTMENT, HARYANA | 2026-07-09</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-2d7fabd90086/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-47bdf7690092/publicNotice</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -2901,34 +2901,34 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>NOTICE REGARDING DISPLAY OF OMR ANSWER SHEETS OF THE COMMON ELIGIBILITY TEST (CET)-2025 (GROUP-C) WRITTEN EXAMINATION IN CANDIDATE LOGIN OF ALL APPEARED CANDIDATES | 2026-07-04</t>
+          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR VARIOUS POSTS AGAINST ADVERTISEMENT NO. 06/2026 OF PRISON DEPARTMENT, HARYANA | 2026-07-09</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE REGARDING CONSIDERING CLOSING DATE OF SUBMISSION OF APPLICATION FORM FOR THE POST OF GROUP-D AGAINST ADVERTISEMENT NO. 05/2026. | 2026-07-07</t>
+          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL SCREENING TEST (PST) FOR MALE CONSTABLE (GD) AND MALE CONSTABLE (GOVERNMENT RAILWAY POLICE) AGAINST ADVERTISEMENT NO. 01/2026, CATEGORY NO. 01</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: ai, mis | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-3cc194ce008c/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-47ba32d3008f/publicNotice</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: ai, mis | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE REGARDING CONSIDERING CLOSING DATE OF SUBMISSION OF APPLICATION FORM FOR THE POST OF GROUP-D AGAINST ADVERTISEMENT NO. 05/2026. | 2026-07-07</t>
+          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL SCREENING TEST (PST) FOR MALE CONSTABLE (GD) AND MALE CONSTABLE (GOVERNMENT RAILWAY POLICE) AGAINST ADVERTISEMENT NO. 01/2026, CATEGORY NO. 01 AND 03 OF POLICE DEPARTMENT, HARYANA. | 2026-07-09</t>
         </is>
       </c>
     </row>
@@ -8645,8 +8645,635 @@
         </is>
       </c>
     </row>
+    <row r="136" ht="30" customHeight="1">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Skip to Main Content</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr"/>
+      <c r="D136" s="2" t="inlineStr"/>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx#data</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>Skip to Main Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="30" customHeight="1">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Vision &amp; Mission</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr"/>
+      <c r="D137" s="2" t="inlineStr"/>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=2UwI/bnoe0Bk6sAjqEVqwQ==</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L137" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>Vision &amp; Mission</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="30" customHeight="1">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Commission &amp; Incumbency Chart</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr"/>
+      <c r="D138" s="2" t="inlineStr"/>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=ZJj9IBSdU7Y1yw0WvPyFPw==</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>Commission &amp; Incumbency Chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="30" customHeight="1">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>Download Admission Certificate</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr"/>
+      <c r="D139" s="2" t="inlineStr"/>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>javascript:__doPostBack('ctl00$generic_masterpage1$ctl15','')</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>Download Admission Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="30" customHeight="1">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Advertisements</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr"/>
+      <c r="D140" s="2" t="inlineStr"/>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=MeNGKau42B9VX4Nn6oZfXA==</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>Advertisements</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="30" customHeight="1">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr"/>
+      <c r="D141" s="2" t="inlineStr"/>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=iQvy8ONZ1XeCyxFZaY2SfA==</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Download Admission Certificate</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr"/>
+      <c r="D142" s="2" t="inlineStr"/>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=VO/uz97buK3DBoFIVkTEOw==</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>Download Admission Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="30" customHeight="1">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Transparency &amp; Objectivity</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr"/>
+      <c r="D143" s="2" t="inlineStr"/>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=jWDzPJrrf4pbXjUrVhA7Hg==</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>Transparency &amp; Objectivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Recruitment Calendar</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr"/>
+      <c r="D144" s="2" t="inlineStr"/>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=N5n/48rKoj1sNGZtqat51w==</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>Recruitment Calendar</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Attestation &amp; Bio Data Form</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: data | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr"/>
+      <c r="D145" s="2" t="inlineStr"/>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=M4ZLp2jMx/L7RLr5Gfi2Eg==</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: data | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>Attestation &amp; Bio Data Form</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Usage Terms &amp; Conditions</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr"/>
+      <c r="D146" s="2" t="inlineStr"/>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=wmpmoV8VNcfB9LTvZnxjTQ==</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>Usage Terms &amp; Conditions</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M135"/>
+  <autoFilter ref="A1:M146"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8657,7 +9284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M136"/>
+  <dimension ref="A1:M147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -9372,7 +9999,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Regular)-2025 Advt.No.-01/2026 (02-07-2026)</t>
+          <t>Press release and written result of the Recruitment of Forest Range Officer,Advt.No.-04/2024 (03-07-2026)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -9382,17 +10009,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>02-07-2026</t>
+          <t>03-07-2026</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>02-07-2026</t>
+          <t>03-07-2026</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_and_P.T_Result_01_26_dated_02_07_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_and_Written_Result_04_24_dated_03_07_2026.pdf</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -9430,44 +10057,44 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Regular)-2025 Advt.No.-01/2026 (02-07-2026)</t>
+          <t>Press release and written result of the Recruitment of Forest Range Officer,Advt.No.-04/2024 (03-07-2026)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Press release and written result of the Recruitment of Forest Range Officer,Advt.No.-04/2024 (03-07-2026)</t>
+          <t>Examination | Combined State/Upper Subordinate Services Examination | | A-1/E-1/2026 , 25/06/2026 | 25/06/2026 | 27/07/2026 | 27/07/2026 | 03/08/2026 | 25/06/2026 03/08/2026 | User</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>03-07-2026</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>03-07-2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_and_Written_Result_04_24_dated_03_07_2026.pdf</t>
+          <t>https://uppsc.up.nic.in/OuterPages/UserHelp.aspx?ID=114</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Uttar Pradesh</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>JPSC</t>
+          <t>UPPSC</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -9485,54 +10112,54 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/</t>
+          <t>https://uppsc.up.nic.in/CandidatePages/Notifications.aspx</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Press release and written result of the Recruitment of Forest Range Officer,Advt.No.-04/2024 (03-07-2026)</t>
+          <t>Examination | Combined State/Upper Subordinate Services Examination | | A-1/E-1/2026 , 25/06/2026 | 25/06/2026 | 27/07/2026 | 27/07/2026 | 03/08/2026 | 25/06/2026 03/08/2026 | User Instructions | View Advertisement | Apply</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Examination | Combined State/Upper Subordinate Services Examination | | A-1/E-1/2026 , 25/06/2026 | 25/06/2026 | 27/07/2026 | 27/07/2026 | 03/08/2026 | 25/06/2026 03/08/2026 | User</t>
+          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 (06-07-2026)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Education/subject not clearly matched</t>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>06-07-2026</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>06-07-2026</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://uppsc.up.nic.in/OuterPages/UserHelp.aspx?ID=114</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_and_P.T_Result_05_26_dated_06_07_2026.pdf</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Uttar Pradesh</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>UPPSC</t>
+          <t>JPSC</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -9550,44 +10177,44 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Education/subject not clearly matched</t>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>https://uppsc.up.nic.in/CandidatePages/Notifications.aspx</t>
+          <t>https://www.jpsc.gov.in/</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Examination | Combined State/Upper Subordinate Services Examination | | A-1/E-1/2026 , 25/06/2026 | 25/06/2026 | 27/07/2026 | 27/07/2026 | 03/08/2026 | 25/06/2026 03/08/2026 | User Instructions | View Advertisement | Apply</t>
+          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 (06-07-2026)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 (06-07-2026)</t>
+          <t>Press Release regarding Combined Civil Services Main Examination Uploaded date:-07-07-2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>06-07-2026</t>
+          <t>07-07-2026</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>06-07-2026</t>
+          <t>07-07-2026</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_and_P.T_Result_05_26_dated_06_07_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_05_26_dated_07_07_2026.pdf</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -9615,7 +10242,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -9625,19 +10252,19 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Press release and P.T. result of the Recruitment of Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 (06-07-2026)</t>
+          <t>Press Release regarding Combined Civil Services Main Examination Uploaded date:-07-07-2026</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Press Release regarding Combined Civil Services Main Examination Uploaded date:-07-07-2026</t>
+          <t>Press release and written result of the Recruitment of Assistant Conservator of Forest,Advt.No.-03/2024 (07-07-2026)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -9652,7 +10279,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_05_26_dated_07_07_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_and_Written_Result_03_24_dated_07_07_2026.pdf</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -9667,7 +10294,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>General/Other</t>
+          <t>Office/Clerical</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
@@ -9680,7 +10307,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -9690,34 +10317,34 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Press Release regarding Combined Civil Services Main Examination Uploaded date:-07-07-2026</t>
+          <t>Press release and written result of the Recruitment of Assistant Conservator of Forest,Advt.No.-03/2024 (07-07-2026)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Press release and written result of the Recruitment of Assistant Conservator of Forest,Advt.No.-03/2024 (07-07-2026)</t>
+          <t>Press Release regarding Recruitment of Deputy Director, Prosecution Advt.No.-15/2023 Uploaded date:-08-12-2025</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Specific non-CSE subject appears required | Non-CSE subject risk: prosecution | Last date appears closed</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>07-07-2026</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>07-07-2026</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_and_Written_Result_03_24_dated_07_07_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_15_23_dated_08_12_2025.pdf</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -9732,7 +10359,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Office/Clerical</t>
+          <t>General/Other</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
@@ -9745,7 +10372,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: it  | Specific non-CSE subject appears required | Non-CSE subject risk: prosecution | Last date appears closed</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -9755,34 +10382,34 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Press release and written result of the Recruitment of Assistant Conservator of Forest,Advt.No.-03/2024 (07-07-2026)</t>
+          <t>Press Release regarding Recruitment of Deputy Director, Prosecution Advt.No.-15/2023 Uploaded date:-08-12-2025</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Press Release regarding Recruitment of Deputy Director, Prosecution Advt.No.-15/2023 Uploaded date:-08-12-2025</t>
+          <t>Press release and Instructions regarding Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 uploaded date :09-05-2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Specific non-CSE subject appears required | Non-CSE subject risk: prosecution | Last date appears closed</t>
+          <t>Auto-extracted: Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-05-2026</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-05-2026</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_15_23_dated_08_12_2025.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_05_26_dated_09_05_2026.pdf</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -9810,7 +10437,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Specific non-CSE subject appears required | Non-CSE subject risk: prosecution | Last date appears closed</t>
+          <t>Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -9820,34 +10447,34 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Press Release regarding Recruitment of Deputy Director, Prosecution Advt.No.-15/2023 Uploaded date:-08-12-2025</t>
+          <t>Press release and Instructions regarding Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 uploaded date :09-05-2026</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Press release and Instructions regarding Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 uploaded date :09-05-2026</t>
+          <t>Press release regarding Jharkhand Combined Civil Services Examination, Advt.No.-01/2026, 05/2026 and 06/2026 (09-07-2026)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>09-05-2026</t>
+          <t>09-07-2026</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>09-05-2026</t>
+          <t>09-07-2026</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.jpsc.gov.in/data/Press_Release_05_26_dated_09_05_2026.pdf</t>
+          <t>https://www.jpsc.gov.in/data/Press_Release_06_26_dated_09_07_2026.pdf</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -9875,7 +10502,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Education/subject not clearly matched | Last date appears closed</t>
+          <t>Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -9885,7 +10512,7 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Press release and Instructions regarding Jharkhand Combined Civil Services Examination (Backlog)-2025 Advt.No.-05/2026 uploaded date :09-05-2026</t>
+          <t>Press release regarding Jharkhand Combined Civil Services Examination, Advt.No.-01/2026, 05/2026 and 06/2026 (09-07-2026)</t>
         </is>
       </c>
     </row>
@@ -10672,7 +11299,7 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 01/2026, 02/2026 &amp; 04/</t>
+          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 02/2026 &amp; 04/2026 | 20</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -10682,17 +11309,17 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-0506603f0071/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-23d707fe007d/publicNotice</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -10730,34 +11357,34 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 01/2026, 02/2026 &amp; 04/2026 | 2026-06-26</t>
+          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 02/2026 &amp; 04/2026 | 2026-07-02</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 02/2026 &amp; 04/2026 | 20</t>
+          <t>NOTICE REGARDING DISPLAY OF OMR ANSWER SHEETS OF THE COMMON ELIGIBILITY TEST (CET)-2025 (GROUP-C) WRITTEN EXAMINATION IN CANDIDATE LOGIN OF ALL APPEARED CANDIDATES | 2026-07-04</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-23d707fe007d/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-2d7fabd90086/publicNotice</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -10785,7 +11412,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -10795,34 +11422,34 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE TO THE ABSENTEE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR THE VARIOUS POSTS OF VARIOUS DEPARTMENTS AGAINST ADVERTISEMENT NOS. 13/2024, 02/2026 &amp; 04/2026 | 2026-07-02</t>
+          <t>NOTICE REGARDING DISPLAY OF OMR ANSWER SHEETS OF THE COMMON ELIGIBILITY TEST (CET)-2025 (GROUP-C) WRITTEN EXAMINATION IN CANDIDATE LOGIN OF ALL APPEARED CANDIDATES | 2026-07-04</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL SCREENING TEST (PST) FOR MALE CONSTABLE (GD) AND MALE CONSTABLE (GOVERNMENT RAILWAY POLICE) AGAINST ADVERTISEMENT NO. 01/2026, CATEGORY NO. 01</t>
+          <t>PUBLIC NOTICE REGARDING CONSIDERING CLOSING DATE OF SUBMISSION OF APPLICATION FORM FOR THE POST OF GROUP-D AGAINST ADVERTISEMENT NO. 05/2026. | 2026-07-07</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: ai, mis | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-237201a5007a/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-3cc194ce008c/publicNotice</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -10850,7 +11477,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: ai, mis | Education/subject not clearly matched | Last date appears closed</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -10860,34 +11487,34 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL SCREENING TEST (PST) FOR MALE CONSTABLE (GD) AND MALE CONSTABLE (GOVERNMENT RAILWAY POLICE) AGAINST ADVERTISEMENT NO. 01/2026, CATEGORY NO. 01 AND 03 OF POLICE DEPARTMENT, HARYANA. | 2026-07-02</t>
+          <t>PUBLIC NOTICE REGARDING CONSIDERING CLOSING DATE OF SUBMISSION OF APPLICATION FORM FOR THE POST OF GROUP-D AGAINST ADVERTISEMENT NO. 05/2026. | 2026-07-07</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>NOTICE REGARDING DISPLAY OF OMR ANSWER SHEETS OF THE COMMON ELIGIBILITY TEST (CET)-2025 (GROUP-C) WRITTEN EXAMINATION IN CANDIDATE LOGIN OF ALL APPEARED CANDIDATES | 2026-07-04</t>
+          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR VARIOUS POSTS AGAINST ADVERTISEMENT NO. 06/2026 OF PRISON DEPARTMENT, HARYANA | 2026-07-09</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-2d7fabd90086/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-47bdf7690092/publicNotice</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -10915,7 +11542,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -10925,34 +11552,34 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>NOTICE REGARDING DISPLAY OF OMR ANSWER SHEETS OF THE COMMON ELIGIBILITY TEST (CET)-2025 (GROUP-C) WRITTEN EXAMINATION IN CANDIDATE LOGIN OF ALL APPEARED CANDIDATES | 2026-07-04</t>
+          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL MEASUREMENT TEST (PMT) FOR VARIOUS POSTS AGAINST ADVERTISEMENT NO. 06/2026 OF PRISON DEPARTMENT, HARYANA | 2026-07-09</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE REGARDING CONSIDERING CLOSING DATE OF SUBMISSION OF APPLICATION FORM FOR THE POST OF GROUP-D AGAINST ADVERTISEMENT NO. 05/2026. | 2026-07-07</t>
+          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL SCREENING TEST (PST) FOR MALE CONSTABLE (GD) AND MALE CONSTABLE (GOVERNMENT RAILWAY POLICE) AGAINST ADVERTISEMENT NO. 01/2026, CATEGORY NO. 01</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Auto-extracted: Computer/IT/office keywords: ai, mis | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-3cc194ce008c/publicNotice</t>
+          <t>https://hssc.gov.in/file/ac1f23cd-9d9c-1328-819f-47ba32d3008f/publicNotice</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -10980,7 +11607,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Computer/IT/office keywords: ai, mis | Education/subject not clearly matched | Last date appears closed</t>
+          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -10990,7 +11617,7 @@
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC NOTICE REGARDING CONSIDERING CLOSING DATE OF SUBMISSION OF APPLICATION FORM FOR THE POST OF GROUP-D AGAINST ADVERTISEMENT NO. 05/2026. | 2026-07-07</t>
+          <t>NOTICE TO THE CANDIDATES FOR PHYSICAL SCREENING TEST (PST) FOR MALE CONSTABLE (GD) AND MALE CONSTABLE (GOVERNMENT RAILWAY POLICE) AGAINST ADVERTISEMENT NO. 01/2026, CATEGORY NO. 01 AND 03 OF POLICE DEPARTMENT, HARYANA. | 2026-07-09</t>
         </is>
       </c>
     </row>
@@ -16669,8 +17296,635 @@
         </is>
       </c>
     </row>
+    <row r="137" ht="30" customHeight="1">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Skip to Main Content</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr"/>
+      <c r="D137" s="2" t="inlineStr"/>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx#data</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: ai | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L137" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>Skip to Main Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="30" customHeight="1">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Vision &amp; Mission</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr"/>
+      <c r="D138" s="2" t="inlineStr"/>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=2UwI/bnoe0Bk6sAjqEVqwQ==</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>Vision &amp; Mission</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="30" customHeight="1">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>Commission &amp; Incumbency Chart</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr"/>
+      <c r="D139" s="2" t="inlineStr"/>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=ZJj9IBSdU7Y1yw0WvPyFPw==</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>Commission &amp; Incumbency Chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="30" customHeight="1">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Download Admission Certificate</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr"/>
+      <c r="D140" s="2" t="inlineStr"/>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>javascript:__doPostBack('ctl00$generic_masterpage1$ctl15','')</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>Download Admission Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="30" customHeight="1">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>Advertisements</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr"/>
+      <c r="D141" s="2" t="inlineStr"/>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=MeNGKau42B9VX4Nn6oZfXA==</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>Advertisements</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr"/>
+      <c r="D142" s="2" t="inlineStr"/>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=iQvy8ONZ1XeCyxFZaY2SfA==</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="30" customHeight="1">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Download Admission Certificate</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr"/>
+      <c r="D143" s="2" t="inlineStr"/>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=VO/uz97buK3DBoFIVkTEOw==</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: mis | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>Download Admission Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Transparency &amp; Objectivity</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr"/>
+      <c r="D144" s="2" t="inlineStr"/>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=jWDzPJrrf4pbXjUrVhA7Hg==</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>Transparency &amp; Objectivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Recruitment Calendar</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr"/>
+      <c r="D145" s="2" t="inlineStr"/>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=N5n/48rKoj1sNGZtqat51w==</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>Recruitment Calendar</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Attestation &amp; Bio Data Form</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: data | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr"/>
+      <c r="D146" s="2" t="inlineStr"/>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=M4ZLp2jMx/L7RLr5Gfi2Eg==</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: data | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>Attestation &amp; Bio Data Form</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="30" customHeight="1">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>Usage Terms &amp; Conditions</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Auto-extracted: Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr"/>
+      <c r="D147" s="2" t="inlineStr"/>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/Pages/View_Content.aspx?id=wmpmoV8VNcfB9LTvZnxjTQ==</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>OPSC</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>General/Other</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>Avoid or Closed</t>
+        </is>
+      </c>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>Computer/IT/office keywords: it  | Education/subject not clearly matched</t>
+        </is>
+      </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opsc.gov.in/Public/OPSC/Default.aspx</t>
+        </is>
+      </c>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>Usage Terms &amp; Conditions</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M136"/>
+  <autoFilter ref="A1:M147"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>